<commit_message>
created lexicon.xlsl (word variation)
</commit_message>
<xml_diff>
--- a/data/canonical.xlsx
+++ b/data/canonical.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>bangla</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>বদ্দা, কি অবস্থা অঁনোর?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">আপনি ভালো আছেন ম্যাম? </t>
+  </si>
+  <si>
+    <t>অঁনে গম আছন ম্যাম?</t>
   </si>
 </sst>
 </file>
@@ -705,12 +711,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1263,124 +1266,128 @@
       </c>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1" spans="1:2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" ht="25" customHeight="1" spans="1:2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1" spans="1:2">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="25" customHeight="1" spans="1:2">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" ht="25" customHeight="1" spans="1:2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" ht="25" customHeight="1" spans="1:2">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" ht="25" customHeight="1" spans="1:2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" ht="25" customHeight="1" spans="1:2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" ht="25" customHeight="1" spans="1:2">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" ht="25" customHeight="1" spans="1:2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14" ht="25" customHeight="1" spans="1:2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
     </row>
     <row r="15" ht="25" customHeight="1" spans="1:2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
     </row>
     <row r="16" ht="25" customHeight="1" spans="1:2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
     </row>
     <row r="17" ht="25" customHeight="1" spans="1:2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
     </row>
     <row r="18" ht="25" customHeight="1" spans="1:2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
     </row>
     <row r="19" ht="25" customHeight="1" spans="1:2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
     </row>
     <row r="20" ht="25" customHeight="1" spans="1:2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Freeze Canonical Dataset v1.0 (1800 sentence pairs)
</commit_message>
<xml_diff>
--- a/data/canonical.xlsx
+++ b/data/canonical.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3393" uniqueCount="3387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3602" uniqueCount="3596">
   <si>
     <t>bangla</t>
   </si>
@@ -1107,7 +1107,7 @@
     <t>ঢাকায় গিয়ে তো আমাদেরকে ভুলে গেছিস</t>
   </si>
   <si>
-    <t>ঢাহাত যায় রে তো আরারে ভুলি গেইয়্যুস</t>
+    <t>ঢাহাত যায় রে তো আঁরারে ভুলি গেইয়্যুস</t>
   </si>
   <si>
     <t>তুমি আজকে কোথায় গিয়েছিলে?</t>
@@ -2811,7 +2811,7 @@
     <t>দরজা খুলে দেখি একটা সুন্দরী মেয়ে দাঁড়িয়ে আছে</t>
   </si>
   <si>
-    <t>দরজা খুলি দেহি উজ্ঞো সুন্দরী মাইফুয়া থিয়েই আছে</t>
+    <t>দরজা খুলি দেহি উজ্ঞো সুন্দরী মেইফুওয়া থিয়েই আছে</t>
   </si>
   <si>
     <t>দরজার বাইরে একটা ভিক্কুক দাঁড়ায় আছে, চাল গুলো উনাকে দিয়ে আসো</t>
@@ -3903,7 +3903,7 @@
     <t>গ্রামের মেয়েরা হাঁস মুরগি পালন করে</t>
   </si>
   <si>
-    <t>গ্রামোর মাইফুয়া অক্কলে আঁস কুরো ফালে</t>
+    <t>গ্রামোর মেইফুওয়া অক্কলে আঁস কুরো ফালে</t>
   </si>
   <si>
     <t>পুকুরে অনেক বড় একটা শোল মাছ দেখেছি</t>
@@ -4011,7 +4011,7 @@
     <t>মেয়েটা একদম তার মায়ের মতো হয়েছে</t>
   </si>
   <si>
-    <t>মাইফুয়া একদম ইতির মা'র মতন অইয়্যি</t>
+    <t>মেইফুওয়া একদম ইতির মা'র মতন অইয়্যি</t>
   </si>
   <si>
     <t>স্বভাব চরিত্র তো সব তোর ভাইয়ের মতো হয়েছে</t>
@@ -4675,7 +4675,7 @@
     <t>পাশের বাড়ির মেয়েগুলো প্রতিদিন আমাদের পেয়ারা গাছ থেকে পেয়ারা চুরি করে</t>
   </si>
   <si>
-    <t>পাশোর বারির মাইফুয়া এগুন আঁরো গুয়াসি গাছুত্তুন গুয়াছি চুরি গরে</t>
+    <t>পাশোর বারির মেইফুওয়া এগুন আঁরো গুয়াসি গাছুত্তুন গুয়াছি চুরি গরে</t>
   </si>
   <si>
     <t>ওদেরকে একবার আমার বড় আপু অনেক বকা দিয়েছিল</t>
@@ -4993,7 +4993,7 @@
     <t>চাচি, আপনার ছেলে-মেয়ে কয়টা?</t>
   </si>
   <si>
-    <t>চাচি, অঁনোর ফোওয়া-মাইফুয়া হওয়ো?</t>
+    <t>চাচি, অঁনোর ফোওয়া-মেইফুওয়া হওয়ো?</t>
   </si>
   <si>
     <t>এটা এরকম হয়ে যাবে যে সেটা আমি আগে বুঝতে পারিনি</t>
@@ -5407,7 +5407,7 @@
     <t>আমার মনে হচ্ছে মেয়েটা তোকে যাদু করেছে</t>
   </si>
   <si>
-    <t>আত্তুন মনে অদ্দে মাইফুয়া ইবে তুরে যাদু গইজ্জি</t>
+    <t>আত্তুন মনে অদ্দে মেইফুওয়া ইবে তুরে যাদু গইজ্জি</t>
   </si>
   <si>
     <t>যদি যাদু না করত, তাহলে তুই এরকম পাগল হয়ে যেতি না</t>
@@ -5761,7 +5761,7 @@
     <t>মেয়েটা হাত মোজা পড়েছিল</t>
   </si>
   <si>
-    <t>মাইফুয়া ইবে আত মৌজো ফইজ্জিল</t>
+    <t>মেইফুওয়া ইবে আত মৌজো ফইজ্জিল</t>
   </si>
   <si>
     <t>প্যান্টটা আমার লম্বা হবে</t>
@@ -6982,7 +6982,7 @@
     <t>ছেলেমেয়ে একসাথে দূরে ঘুরতে যাওয়া ঠিক না</t>
   </si>
   <si>
-    <t>ফোওয়া-মাইফুয়া একলগে দুরে ঘুইত্তু যন ঠিক ন</t>
+    <t>ফোওয়া-মেইফুওয়া একলগে দুরে ঘুইত্তু যন ঠিক ন</t>
   </si>
   <si>
     <t>আমি সবাইকে ফোন করে দিয়েছি, কিছুক্ষণের মধ্যে সবাই চলে আসবে</t>
@@ -9214,7 +9214,7 @@
     <t>মেয়েটার সারারাত জ্বর ছিল, কিছু খেতে পারেনি</t>
   </si>
   <si>
-    <t>মাইফুয়া ইবের আরা রাইত জ্বর আছিল, কিছু হাইত ন পারে</t>
+    <t>মেইফুওয়া ইবের আরা রাইত জ্বর আছিল, কিছু হাইত ন পারে</t>
   </si>
   <si>
     <t>পায়ে খুব ব্যথা করছে, একটু টিপে দাও তো</t>
@@ -9604,7 +9604,7 @@
     <t>এই মেয়েটা থেকে দূরে থাকিস, এর মতিগতি ভালো না</t>
   </si>
   <si>
-    <t>এই মাইফোওয়া ইবেত্তুন দূরে থাহিস, ইবের মতিগতি ভালা নো</t>
+    <t>এই মেইফুওয়া ইবেত্তুন দূরে থাহিস, ইবের মতিগতি ভালা নো</t>
   </si>
   <si>
     <t>তোমাকে আমি অনেক বিশ্বাস করি, দয়া করে এমন করো না</t>
@@ -9892,7 +9892,7 @@
     <t>আমাদের পথ এখানেই শেষ না, আজ হেরে গেছি তো কী হয়েছে</t>
   </si>
   <si>
-    <t>আরার পথ এনডেই শেষ নো, আজিয়ে অডি গেই তো কী অইয়্যি</t>
+    <t>আঁরার পথ এনডেই শেষ নো, আজিয়ে অডি গেই তো কী অইয়্যি</t>
   </si>
   <si>
     <t>তুই এগুলো নিয়েছিস কত দিন হচ্ছে?</t>
@@ -9902,6 +9902,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="SolaimanLipi"/>
+        <charset val="134"/>
+      </rPr>
       <t>আমার তো ঠিকমতো মনে নেই, মনে হয় ১৫</t>
     </r>
     <r>
@@ -9996,7 +10002,7 @@
     <t>তোমার সাহস তো কম না, তুমি অন্য গ্রামের হয়ে এই গ্রামের মেয়েকে ডিস্টার্ব করো!</t>
   </si>
   <si>
-    <t>তোঁয়ার সাহস তো হম নো, তুঁই অন্য গ্রামুর অইয়্যিরে এই গ্রামুর মাইফোয়ারে ডিস্টার্ব গরো!</t>
+    <t>তোঁয়ার সাহস তো হম নো, তুঁই অন্য গ্রামুর অইয়্যিরে এই গ্রামুর মেইফুওয়ারে ডিস্টার্ব গরো!</t>
   </si>
   <si>
     <t>যদি ঝামেলা করতে না চাও, তাহলে এখনই এখান থেকে চলে যাও</t>
@@ -10284,34 +10290,661 @@
     <t>সবাই সামনে থেকে সরে দাঁড়ান, ট্রাক আসছে</t>
   </si>
   <si>
+    <t>বিয়াজ্ঞুন সামনুত্তুন সরি থিয়ন, টেরাক আইয়্যির</t>
+  </si>
+  <si>
     <t>বাবা, তোমার সঙ্গে আমার কিছু কথা আছে</t>
   </si>
   <si>
+    <t>বাবা, তোঁয়ার লগে আঁর কিছু হতা আছিল</t>
+  </si>
+  <si>
     <t>আমি সারাদিন না খেয়ে আছি, আমাকে কিছু খেতে দিন</t>
   </si>
   <si>
+    <t>আঁই আরাদিন ন হায় আছি, আঁরে কিছু হাইতু দন</t>
+  </si>
+  <si>
     <t>আম্মু, একটু কষ্ট করে আমার ঘরটা গুছিয়ে দাও, বিকেলে মেহমান আসবে</t>
   </si>
   <si>
+    <t>আম্মু, এক্কানা হষ্ট গরি আঁর ঘরগান গুছায় দও, বিকেলে মেমাম আইবু</t>
+  </si>
+  <si>
     <t>আম্মু, আমার বন্ধু বাড়িতে আসবে, আজ একটু ভালো কিছু রান্না করো</t>
   </si>
   <si>
+    <t>আম্মু, আঁর বন্ধু বারিত আইবু, আজিয়ে এক্কানা ভালা কিছু রান্না গরো</t>
+  </si>
+  <si>
     <t>মা, আজ একটু আগে রান্না করো, বাবার অফিসে যেতে দেরি হয়ে যাচ্ছে</t>
   </si>
   <si>
+    <t>মা, আজিয়ে এক্কানা আগে রান্না গরো, বাবার অফিসুত যাইতে দেরি অই যার</t>
+  </si>
+  <si>
     <t>স্যার, আমার আবেদনটা একটু ওপরে পাঠিয়ে দিন, অনেক দিন ধরে আটকে আছে</t>
   </si>
   <si>
+    <t>স্যার, আঁর আবেদন ইয়েন এক্কানা উরে পাঠাই দন, বতদিন ধরি আটকি আছে</t>
+  </si>
+  <si>
     <t>ভাই, প্লিজ রাস্তার মাঝখানে গাড়ি না রেখে পাশে সরিয়ে নিন</t>
   </si>
   <si>
+    <t>বদ্দা, প্লিজ রাস্তার মাঝে গারি ন রাহি পাশে সরাই লন</t>
+  </si>
+  <si>
     <t>বাবা, আমার সাইকেলটা একটু মেরামত করিয়ে দাও, চাকা নষ্ট হয়ে গেছে</t>
   </si>
   <si>
+    <t>বাবা, আঁর সাইকেলগান এক্কানা মেরামত গরাই দও, চাক্কা নষ্ট অই গেইয়্যি</t>
+  </si>
+  <si>
     <t>আম্মু, আমার জন্য একটু শরবত বানিয়ে দাও, অনেক গরম লাগছে</t>
   </si>
   <si>
+    <t>আম্মু, আঁর লাই এক্কানা শরবত বানাই দও, বত গরম লাগের</t>
+  </si>
+  <si>
     <t>আমি হিসাব করে দেখিনি কত টাকা আছে</t>
+  </si>
+  <si>
+    <t>আঁই হিসেব গরি ন চায় হতো টিয়া আছে</t>
+  </si>
+  <si>
+    <t>একটু হাত লাগান, আপনি ছাড়া এটা ওপরে তোলা সম্ভব না</t>
+  </si>
+  <si>
+    <t>এক্কানা আত লাগন, অঁনে ছারা ইয়েন উরে তোলন সম্ভব নো</t>
+  </si>
+  <si>
+    <t>সায়েমকে ফোন করে জিজ্ঞেস কর, পরীক্ষা কখন সেটা</t>
+  </si>
+  <si>
+    <t>সায়েম উরে ফোন গরি ফুস গর, পরীক্ষে হত্তে ইয়েন</t>
+  </si>
+  <si>
+    <t>স্যার, পরীক্ষায় এই প্রশ্নটা আসবে কি না একটু বলবেন?</t>
+  </si>
+  <si>
+    <t>স্যার, পরীক্ষেত এই প্রশ্ন ইয়েন আইবু কিনা এক্কানা হইবেন?</t>
+  </si>
+  <si>
+    <t>আজ ক্লাসে যা পড়িয়েছে, সব আমার মাথার ওপর দিয়ে গেছে</t>
+  </si>
+  <si>
+    <t>আজিয়ে ক্লাসুত যা পরাইয়্যি বিয়াক আঁর মাথার উদ্দি গেইয়্যি</t>
+  </si>
+  <si>
+    <t>নতুন স্যারের পড়াগুলো কিছু বুঝি না</t>
+  </si>
+  <si>
+    <t>নতুন স্যার উর পরা এগিন কিছু ন বুঝির</t>
+  </si>
+  <si>
+    <t>আমার তো উনার ক্লাস করলে ঘুম চলে আসে</t>
+  </si>
+  <si>
+    <t>আত্তুন তো ইবের ক্লাস গরিলি ঘুম চলি আইয়্যি</t>
+  </si>
+  <si>
+    <t>জামিল স্যারের ক্লাসে আমার খুব বিরক্ত লাগে, কী পড়ান আগামাথা বুঝি না</t>
+  </si>
+  <si>
+    <t>জামিল স্যার উর ক্লাসুত আঁর খুব বিরক্ত লাগে, কি পরাই আগামাথা ন বুঝি</t>
+  </si>
+  <si>
+    <t>স্যার, কোন টপিকগুলো পরীক্ষায় আসবে যদি বলতেন</t>
+  </si>
+  <si>
+    <t>স্যার, হন টপিকগিন পরীক্ষেত আইবু যদি হইতেন</t>
+  </si>
+  <si>
+    <t>অফিসের নতুন কলিগটা অনেক মিশুক, সবার সঙ্গে খুব তাড়াতাড়ি মিশে যাচ্ছে</t>
+  </si>
+  <si>
+    <t>আফিসুর নতুন কলিগ ইবে বত মিশুক, বিয়াজ্ঞুনুর লগে বত তারাতারি মিশি যার</t>
+  </si>
+  <si>
+    <t>ম্যাম, আমার বন্ধু অসুস্থ, তাই আজ ক্লাস করতে পারেনি</t>
+  </si>
+  <si>
+    <t>ম্যাম, আঁর বন্ধু অসুস্থ, এতেল্লে আজিয়ে ক্লাস গরিত নো পারে</t>
+  </si>
+  <si>
+    <t>অফিসে নতুন সফটওয়্যার এসেছে, ওটা ব্যবহার করতে সমস্যা হচ্ছে</t>
+  </si>
+  <si>
+    <t>অফিসুত নতুন সফটওয়্যার আইসসি, ইবে বেবার গত্তে সমস্যা অর</t>
+  </si>
+  <si>
+    <t>ঝড় তো থামার নাম নিচ্ছে না, একটানা পড়েই যাচ্ছে</t>
+  </si>
+  <si>
+    <t>ঝর তো থামিবের নাম ন লর, একটানা পরিই যার</t>
+  </si>
+  <si>
+    <t>এভাবে আর কয়েক দিন বৃষ্টি পড়লে মাঠের সব ফসল নষ্ট হয়ে যাবে</t>
+  </si>
+  <si>
+    <t>এন গরি আর হয়েকদিন ঝর ফরিলি মাডোর বিয়াক ফসল নষ্ট অই যাইবু</t>
+  </si>
+  <si>
+    <t>আজ কলিগের সাথে একটু ভুল-বোঝাবুঝি হয়েছে, তাই একটু মুড অফ</t>
+  </si>
+  <si>
+    <t>আজিয়ে কলিগুর লগে এক্কানা ভুল বোঝাবুঝি অইয়্যি, এতেল্লে এক্কানা মুড অফ</t>
+  </si>
+  <si>
+    <t>স্যার, আপনি বলেছিলেন ক্লাস টেস্ট না নিয়ে অ্যাসাইনমেন্ট দেবেন</t>
+  </si>
+  <si>
+    <t>স্যার, অঁনে হইলেন ক্লাস টেস্ট ন লই অ্যাসাইনমেন্ট দিবেন</t>
+  </si>
+  <si>
+    <t>আজ অ্যাসাইনমেন্ট জমা দেওয়ার শেষ দিন</t>
+  </si>
+  <si>
+    <t>আজিয়ে অ্যাসাইনমেন্ট জমা দিবের শেষ দিন</t>
+  </si>
+  <si>
+    <t>গতবার আমাদের প্রশ্ন অনেক কঠিন হয়েছিল, তাই এবার সহজ হতে হবে</t>
+  </si>
+  <si>
+    <t>গতবার আঁরার প্রশ্ন বত কঠিন অইয়্যিল, এতেল্লে এবার সহজ অন ফরিবু</t>
+  </si>
+  <si>
+    <t>স্যার, ক্লাস টেস্টের ফলাফল কবে দেবেন, অনেক দিন ধরে অপেক্ষা করছি</t>
+  </si>
+  <si>
+    <t>স্যার, ক্লাস টেস্ট উর ফলাফল হত্তে দিবেন, বত দিন ধরি অপেক্ষা গরির</t>
+  </si>
+  <si>
+    <t>তোর বাবাকে ফোন করে বল তাড়াতাড়ি চলে আসতে</t>
+  </si>
+  <si>
+    <t>তোর বাফুরে ফোন গরি হ হারা চলি আইসতু</t>
+  </si>
+  <si>
+    <t>লিখতে লিখতে আমার হাত ব্যথা হয়ে গেছে, তাও লেখা শেষ হয় না</t>
+  </si>
+  <si>
+    <t>লেখতে লেখতে আঁর আত ব্যথা অই গেইয়্যি, তাও লেহা শেষ ন অর</t>
+  </si>
+  <si>
+    <t>স্যার, আমি ওর দিকে তাকাইনি</t>
+  </si>
+  <si>
+    <t>স্যার, আঁই ইতের মিক্কে নো চাই</t>
+  </si>
+  <si>
+    <t>পরীক্ষার হলে যদি শব্দ করো, তাহলে সবার খাতা নিয়ে ফেলব</t>
+  </si>
+  <si>
+    <t>পরীক্ষের হলুত যদি শব্দ গরো, তইলি বিয়াজ্ঞুনুর হাতা লই ফেলাইয়্যুম</t>
+  </si>
+  <si>
+    <t>স্যার, আমার খাতা নেবেন না, আমি ওর থেকে দেখিনি</t>
+  </si>
+  <si>
+    <t>স্যার, আঁর হাতা ন লইয়্যুন, আঁই ইতেত্তুন নো চাই</t>
+  </si>
+  <si>
+    <t>কপি করলে করো, কিন্তু শব্দ করবে না</t>
+  </si>
+  <si>
+    <t>কপি গরিলি গরো, কিন্তু শব্দ ন গইজ্জো</t>
+  </si>
+  <si>
+    <t>স্যার, অনেকক্ষণ হয়ে গেল, এবার যদি আমার খাতাটা দিয়ে দিতেন</t>
+  </si>
+  <si>
+    <t>স্যার, বত হতক্ষন অই গেইয়্যি, এবার যদি আঁর হাতাগো দি দিতেন</t>
+  </si>
+  <si>
+    <t>ম্যাম, এমনটা আর হবে না, সত্যি বলছি</t>
+  </si>
+  <si>
+    <t>ম্যাম, এল্লেত আর ন অইবু, সত্যি হইদ্দি</t>
+  </si>
+  <si>
+    <t>আমি তোর থেকে দেখব, আর তুই রিফার থেকে দেখিস</t>
+  </si>
+  <si>
+    <t>আঁই তোত্তুন চাইয়্যুম, আর তুই রিফাত্তুন চাইস</t>
+  </si>
+  <si>
+    <t>আমি এখান থেকে দেখতে পারছি না, তুই খাতাটা আরেকটু উঁচু করে ধর</t>
+  </si>
+  <si>
+    <t>আঁই এত্তুন ন দেহির, তুই হাতাগো আরেক্কানা উরে গরি ধর</t>
+  </si>
+  <si>
+    <t>একটু সাবধানে, স্যার দেখলে দুজনেরই খাতা নিয়ে ফেলবেন</t>
+  </si>
+  <si>
+    <t>এক্কানা সাবধানে, স্যার দেহিলি দুনুজনুর হাতা লই ফেলাইবু</t>
+  </si>
+  <si>
+    <t>তুই চিন্তা করিস না, স্যার আমাদের কিছু বলবেন না</t>
+  </si>
+  <si>
+    <t>তুই চিন্তে ন গরিস, স্যার আঁরারে কিছু ন হইবু</t>
+  </si>
+  <si>
+    <t>ম্যাম, আমার মা অসুস্থ, তাই গতকাল আসতে পারিনি</t>
+  </si>
+  <si>
+    <t>ম্যাম, আঁর মা অসুস্থ, এতেল্লে গত হালিয়ে আইত ন পারি</t>
+  </si>
+  <si>
+    <t>আজ অফিসে ওভারটাইম করেছি, তাই দেরি হয়ে গেছে</t>
+  </si>
+  <si>
+    <t>আজিয়ে অফিসুত ওভারটাইম গইজ্জি, এতেল্লে দেরি অই গেইয়্যি</t>
+  </si>
+  <si>
+    <t>স্যার, এই অধ্যায়টা পরীক্ষার জন্য কতটা গুরুত্বপূর্ণ বলে মনে করেন?</t>
+  </si>
+  <si>
+    <t>স্যার, এই অধ্যায় ইবে পরীক্ষের লাই হতটা গুরুত্বপূর্ণ বলি মনে গরন?</t>
+  </si>
+  <si>
+    <t>স্যার, পরীক্ষার জন্য কোন কোন অধ্যায় পড়ে যেতে হবে?</t>
+  </si>
+  <si>
+    <t>স্যার, পরীক্ষের লাই হন হন অধ্যায় পরি যন ফরিবু?</t>
+  </si>
+  <si>
+    <t>আমাদের এবার সময় কম, তাই সিলেবাস ছোট রাখলে ভালো হবে</t>
+  </si>
+  <si>
+    <t>আঁরার এবার সময় হম, এতেল্লে সিলেবাস ছোডো রাহিলি ভালা অইবু</t>
+  </si>
+  <si>
+    <t>অফিসের কাজ এত বেশি যে ঘরে ঠিকমতো সময় দিতে পারি না</t>
+  </si>
+  <si>
+    <t>অফিসুর হাজ এব বেশি যে ঘরুত ঠিকমতো সময় দিত ন পারির</t>
+  </si>
+  <si>
+    <t>ম্যাম, পরীক্ষায় ক্যালকুলেটর ব্যবহার করতে পারব?</t>
+  </si>
+  <si>
+    <t>ম্যাম, পরীক্ষেত ক্যালকুলেটর বেবার গরিত ফাইজ্জুম?</t>
+  </si>
+  <si>
+    <t>সবার ব্যাগ আর মোবাইল ফোন সামনে এনে রাখো</t>
+  </si>
+  <si>
+    <t>বিয়াজ্ঞুনুর ব্যাগ আর মোবাইল ফোন সাম্মুদ্দি আনি রাহো</t>
+  </si>
+  <si>
+    <t>যদি পরীক্ষা চলাকালীন কারও কাছে মোবাইল ফোন পাওয়া যায়, তাহলে তাকে হল থেকে বের করে দেওয়া হবে</t>
+  </si>
+  <si>
+    <t>যদি পরীক্ষে চলাকালীন কিয়ার হাছে মোবাইল ফোন পা যায়, তইলি ইতেরে হল উত্তুন বাইর গরি দন অইবু</t>
+  </si>
+  <si>
+    <t>আজ অফিসে একটা ভুল হয়ে গেছে, বসকে কীভাবে বলব বুঝছি না</t>
+  </si>
+  <si>
+    <t>আজিয়ে অফিসুত এক্কান ভুল অই গেইয়্যি, বস উরে কেন গরি হইয়্যুম ন বুঝির</t>
+  </si>
+  <si>
+    <t>ম্যাডাম, পরীক্ষায় উত্তর বাংলায় লিখব, নাকি ইংরেজিতে লিখতে হবে?</t>
+  </si>
+  <si>
+    <t>ম্যাডাম, পরীক্ষেত উত্তর বাংলাত লেইক্কুম নাকি ইংরেজিত লেহন ফরিবু?</t>
+  </si>
+  <si>
+    <t>আমাদের ক্লাসে নতুন একজন ছাত্র ভর্তি হয়েছে</t>
+  </si>
+  <si>
+    <t>আঁরার ক্লাসুত নতুন উজ্ঞো ছাত্র ভর্তি অইয়্যি</t>
+  </si>
+  <si>
+    <t>স্যার, আমি পরীক্ষায় ভালো করতে চাই, কোন বিষয়গুলো বেশি পড়া দরকার?</t>
+  </si>
+  <si>
+    <t>স্যার, আঁই পরীক্ষেত ভালা গইত্তাম চাই, হোন বিষয়গুন বেশি ফরন উর দরহার?</t>
+  </si>
+  <si>
+    <t>আমি তোমাকে আটকে রাখতে চাই না, তোমার চলে যেতে মন চাইলে চলে যেতে পার</t>
+  </si>
+  <si>
+    <t>আঁই তোঁয়ারে আটকাই রাইখতাম ন চাই, তোঁয়াত্তুন চলি যাইতু মন চাইলি চলি যাইত পারো</t>
+  </si>
+  <si>
+    <t>ঘরের অবস্থা ভালো না, পড়াশোনার পাশাপাশি পার্টটাইম কাজ করতে হবে</t>
+  </si>
+  <si>
+    <t>ঘরুর অবস্থা ভালা নো, পরালেহার পাশাপাশি পার্টটাইম হাজ গরন ফরিবু</t>
+  </si>
+  <si>
+    <t>এখানে আরও একটা বিপদ রয়েছে</t>
+  </si>
+  <si>
+    <t>এনডে আরও এক্কান বিপদ আছে</t>
+  </si>
+  <si>
+    <t>কোনো কিছু করার আগে আমাদেরকে এখান থেকে বের হতে হবে</t>
+  </si>
+  <si>
+    <t>হনো কিছু গরিবের আগে আরাত্তুন এত্তুন বাইর অন ফরিবু</t>
+  </si>
+  <si>
+    <t>আমাদের হাতে এখন বেশি সময় নেই, যা করার তাড়াতাড়ি করতে হবে</t>
+  </si>
+  <si>
+    <t>আঁরার আ'তুত এহন বেশি সময় দেইন, যা গরিবের তারাতারি গরন ফরিবু</t>
+  </si>
+  <si>
+    <t>সন্ধ্যার আগে কিছু একটা করতে না পারলে সবাই এখানে আটকা পড়ব</t>
+  </si>
+  <si>
+    <t>আজুইন্নের আগে কিছু এক্কান গরিত ন পারিলি বিয়াজ্ঞুন এনডে আটকি ফইজ্জুম</t>
+  </si>
+  <si>
+    <t>আবির কাঁধে ব্যাগ নিয়ে বের হয়ে গেছে</t>
+  </si>
+  <si>
+    <t>আবির হাধুত ব্যাগ লই বাইর অই গেইয়্যি</t>
+  </si>
+  <si>
+    <t>সে কোথায় গেছে সেটা কি তুমি জানো?</t>
+  </si>
+  <si>
+    <t>ইতে হনডে গেইয়্যি ইয়েন কি তুঁই জানো?</t>
+  </si>
+  <si>
+    <t>যাওয়ার সময় আমাকে কিছু বলে যায়নি</t>
+  </si>
+  <si>
+    <t>যাইবের সমত আঁরে কিছু হই ন যায়</t>
+  </si>
+  <si>
+    <t>কিরে, তোর প্রেমিকার নাকি বিয়ে হয়ে যাচ্ছে?</t>
+  </si>
+  <si>
+    <t>কিরে, তোর প্রেমিকার বলে বিয়ে অই যার?</t>
+  </si>
+  <si>
+    <t>আরে ভাই, এত সিরিয়াস হলে চলবে না, একটু হাসুন</t>
+  </si>
+  <si>
+    <t>আরে বদ্দা, এল্লেত সিরিয়াস অইলি ন চলিবু, এক্কানা আ'সন</t>
+  </si>
+  <si>
+    <t>কিরে, ব্যাপার কী, আজ অনেক হাসিখুশি লাগছে!</t>
+  </si>
+  <si>
+    <t>কিরে, ব্যাপার কী, আজিয়ে বত আ'সিখুশি লাগের!</t>
+  </si>
+  <si>
+    <t>এত হাসিখুশি কেন? বিয়ে ঠিক হলো নাকি?</t>
+  </si>
+  <si>
+    <t>এল্লেত আ'সিখুশি কা? বিয়ে ঠিক অইয়্যি নাকি?</t>
+  </si>
+  <si>
+    <t>আমার সঙ্গে মজা করিস না, আমি এখন মজা করার মুডে নেই</t>
+  </si>
+  <si>
+    <t>আঁর লগে মজা ন গরিস, আঁই এহন মজা গরিবের মুড উত নেই</t>
+  </si>
+  <si>
+    <t>তোর বাবা নাকি আরেকটা বিয়ে করছেন? ঘটনাটা কি সত্যি?</t>
+  </si>
+  <si>
+    <t>তোর বাফ বলে আরেকগো বিয়ে গইজ্জি? ঘটনা ইয়েন কি সত্যি?</t>
+  </si>
+  <si>
+    <t>তোর বউ নাকি পাশের বাড়ির একটা ছেলের সঙ্গে পালিয়ে গেছে?</t>
+  </si>
+  <si>
+    <t>তোর বউ বলে পাশুর বারির ফোওয়ার লগে পালাই গেইয়্যি?</t>
+  </si>
+  <si>
+    <t>কী ব্যাপার! আজ এত সেজেগুজে কোথায় যাচ্ছিস?</t>
+  </si>
+  <si>
+    <t>কী ব্যাপার! আজিয়ে এত সাজিগুজি হনডে যর?</t>
+  </si>
+  <si>
+    <t>এই মেয়েটা তোকে পছন্দ করে মনে হয়</t>
+  </si>
+  <si>
+    <t>এই মেইফুওয়া ইবে তোরে পছন্দ গরে মনে অয়</t>
+  </si>
+  <si>
+    <t>তোমার সঙ্গে কথা বললে সময় যে কখন চলে যায়, বুঝতেই পারি না</t>
+  </si>
+  <si>
+    <t>তোঁয়ার লগে হতা হইলি সময় যে হত্তে চলি যায়, বুঝিতই ন পারি</t>
+  </si>
+  <si>
+    <t>কিরে বাটপার, তোর বাটপারি কেমন চলে?</t>
+  </si>
+  <si>
+    <t>কিরে বাটপার, তোর বাটপারি কেন চলের?</t>
+  </si>
+  <si>
+    <t>তোকে অনেক মিস করছি, তুই না থাকলে কাউকে জ্বালাতে পারি না</t>
+  </si>
+  <si>
+    <t>তোরে বত মিস গইজ্জি, তুই ন থাহিলি কিয়ারে জালাইত ন পারি</t>
+  </si>
+  <si>
+    <t>তোর শুধু বয়সটাই বাড়ছে, কিন্তু বুদ্ধিটা বাড়ছে না</t>
+  </si>
+  <si>
+    <t>তোর উদো বয়সই বেইজ্জি, কিন্তু বুদ্ধি ন বারের</t>
+  </si>
+  <si>
+    <t>ছোটবেলায় যেরকম বেকুব ছিলি, ঠিক এখনো সেরকম বেকুব থেকে গেছিস</t>
+  </si>
+  <si>
+    <t>গুরো থাকতে যেরহম বেকুব আছিলি, ঠিক এহনো সেরহম বেকুব থাহি গেইয়্যুস</t>
+  </si>
+  <si>
+    <t>ভাই, তুই এত খাস কীভাবে, তোরটা পেট নাকি অন্য কিছু!</t>
+  </si>
+  <si>
+    <t>বদ্দা, তুই এত হস কেনে, তোর ইবে পেট নাকি অন্য কিছু!</t>
+  </si>
+  <si>
+    <t>তুই সারাদিন এত এত খাস, তাও মোটা হোস না, আর আমি অল্প খেলেই মোটা হয়ে যাই</t>
+  </si>
+  <si>
+    <t>তুই আরাদিন এত এত হস, তাও মোটা ন অস, আর আঁই অল্প হাইলিই মোটা অই যাই</t>
+  </si>
+  <si>
+    <t>আচ্ছা, তুই যে এত খাস, সেই খাবারগুলো যায় কোথায়?</t>
+  </si>
+  <si>
+    <t>আইচ্ছে, তুই যে এত হস, এই হানা এগিন যায় হনডে?</t>
+  </si>
+  <si>
+    <t>কী রে, তোর চেহারা দেখে মনে হচ্ছে সারারাত ঘুমাসনি</t>
+  </si>
+  <si>
+    <t>কী রে, তোর চিয়ারা দেহি মনে অর আরা রাইত নো ঘুমস</t>
+  </si>
+  <si>
+    <t>সারারাত না ঘুমিয়ে কী করেছিস? কার সঙ্গে কথা বলেছিস?</t>
+  </si>
+  <si>
+    <t>আরা রাইত নো ঘুমাই কি গইজ্জুস? হার লগে হতা হইয়্যুস?</t>
+  </si>
+  <si>
+    <t>কী রে, তুই এখনো সেই পুরোনো অভ্যাস ছাড়তে পারলি না</t>
+  </si>
+  <si>
+    <t>কি রে, তুই এহনো সেই পুরন অভ্যেস ছারিত ন পারিলি</t>
+  </si>
+  <si>
+    <t>আরে, বন্ধু ছাড়া জীবনটা যেন লবণ ছাড়া তরকারির মতো</t>
+  </si>
+  <si>
+    <t>আরে, বন্ধু ছারা জীবন ইয়েন যেন লবণ ছারা তরহারির মতন</t>
+  </si>
+  <si>
+    <t>ভাই, আপনি না এলে আজকের আড্ডাটা একদম জমত না</t>
+  </si>
+  <si>
+    <t>বদ্দা, অঁনে ন আইলি আজিয়ের আড্ডা ইয়েন একদম ন জাইমতো</t>
+  </si>
+  <si>
+    <t>তুই কি সারাজীবন এরকম ছোট থেকে যাবি, নাকি একটু বড় হবি?</t>
+  </si>
+  <si>
+    <t>তুই কি আরা জীবন এরহম ছোডো থাহি যাইবি, নাকি এক্কানা বরো অইবি?</t>
+  </si>
+  <si>
+    <t>এত চিন্তা করলে মাথার চুল যা আছে সব পড়ে যাবে</t>
+  </si>
+  <si>
+    <t>এত চিন্তে গরিলি মাথাত চল যা আছে বিয়াক পরি যাইবু</t>
+  </si>
+  <si>
+    <t>ভাবি, মনে হয় বেশি টেনশন দেই, মাথার চুল তো সব পড়ে যাচ্ছে</t>
+  </si>
+  <si>
+    <t>ভাবি মনে অয় বেশি টেনশন দেই, মাথার চুল তো বিয়াক পরি যার</t>
+  </si>
+  <si>
+    <t>আপনি কি সত্যিই এটা বললেন, নাকি আমি ঘুমের মধ্যে শুনলাম?</t>
+  </si>
+  <si>
+    <t>অঁনে কি সত্যি ইয়েন হইয়্যুন, নাকি আঁই ঘুমুর মধ্যে উইন্নিলাম?</t>
+  </si>
+  <si>
+    <t>আজ সূর্য কোন দিকে উঠছে, তুই আমার বাড়িতে!</t>
+  </si>
+  <si>
+    <t>আজিয়ে সুর্য হুনদি উইট্টি, তুই আঁর বারিত!</t>
+  </si>
+  <si>
+    <t>সবসময় মজা ভালো লাগে না, আমি এখন মজা করার মুডে নেই</t>
+  </si>
+  <si>
+    <t>সবসময় মজা ভালা ন লাগে, আঁই এহন মজা গরিবের মুডুত নেই</t>
+  </si>
+  <si>
+    <t>কিরে, তোর মন কোথায়? কার কাছে চলে গেছে?</t>
+  </si>
+  <si>
+    <t>কিরে, তোর মন হনডে? হার হাছে চলি গেইয়্যি?</t>
+  </si>
+  <si>
+    <t>তোর বয়স বাড়লেও এখনো স্বভাব পরিবর্তন হয়নি</t>
+  </si>
+  <si>
+    <t>তোর বয়স বারিলিও এহনো স্বভাব পরিবর্ত্ন নো অয়</t>
+  </si>
+  <si>
+    <t>সবাই মিলে একটা গান ধর, ভালো লাগবে</t>
+  </si>
+  <si>
+    <t>বিয়াজ্ঞুন মিলি উজ্ঞো গান ধর, ভালা লাগিবু</t>
+  </si>
+  <si>
+    <t>তোর মাথায় মনে হয় কিছু নেই, কিছু থাকলে তো এমন কাজ করতিস না</t>
+  </si>
+  <si>
+    <t>তোর মাথাত মনে অয় কিছু নেই, কিছু থাহিলি তো এরহম হাজ ন গইত্তি</t>
+  </si>
+  <si>
+    <t>তোদের থেকে দূরে থাকলেই ভালো, একসঙ্গে থাকলে একটাও ভালো কথা হয় না</t>
+  </si>
+  <si>
+    <t>তোরাত্তুন দুরে থাহিলিই ভালা, একলগে থাহিলি এক্কানও ভালা হতা নো অয়</t>
+  </si>
+  <si>
+    <t>আমি আগে অনেক ভালো ছিলাম, এখন ওর সঙ্গে মিশতে মিশতে খারাপ হয়ে যাচ্ছি</t>
+  </si>
+  <si>
+    <t>আঁই আগে বত ভালা আছিলাম, এহন ইতের লগে মিশতে মিশতে হারাপ অই যাইর</t>
+  </si>
+  <si>
+    <t>মুখে বলা অনেক সহজ, করে দেখানো অনেক কঠিন</t>
+  </si>
+  <si>
+    <t>মুখে হন বত সোজা, গরি দেহন বত কঠিন</t>
+  </si>
+  <si>
+    <t>এত বকবক না করে কাজে মন দাও, সব কাজ পড়ে আছে</t>
+  </si>
+  <si>
+    <t>এত বকবক ন গরি হাজুত মন দও, বিয়াক হাজ পরি আছে</t>
+  </si>
+  <si>
+    <t>আমি তো তোমার সঙ্গে মজা করছিলাম, তুমি তো দেখি ভয় পেয়ে গেছ</t>
+  </si>
+  <si>
+    <t>আঁই তো তোঁয়ার লগে মজা গরিদ্দি, তুঁই তো দেহি ডরাই গেইয়্যো</t>
+  </si>
+  <si>
+    <t>তোর জন্য মেয়ে খুঁজতে খুঁজতে আমরা সবাই বিরক্ত হয়ে গেছি</t>
+  </si>
+  <si>
+    <t>তোর লাই মেইফুওয়া থোওয়াতে থোওয়াতে আঁরা বিয়াজ্ঞুন বিরক্ত অই গেই</t>
+  </si>
+  <si>
+    <t>মন ভালো থাকলে নাকি আশেপাশের সবকিছু সুন্দর লাগে</t>
+  </si>
+  <si>
+    <t>মন ভালা থাহিলি বলে আশেপাশের বিয়াক কিছু সুন্দর লাগে</t>
+  </si>
+  <si>
+    <t>আজ যে মেয়েটাকে দেখতে গিয়েছিলাম, ওকে ভালো মনে হলো</t>
+  </si>
+  <si>
+    <t>আজিয়ে যে মেইফুওয়ারে চাইতাম গেইলাম, ইবেরে ভালা মনে অইলু</t>
+  </si>
+  <si>
+    <t>যদি মেয়েটা ভালো হয়, তাহলে ওর সঙ্গে কথা বল</t>
+  </si>
+  <si>
+    <t>যদি মেইফুওয়া ইবে ভালা অয়, তইলি ইবের লগে হতা হো</t>
+  </si>
+  <si>
+    <t>আমাদের আরও ভালো করে খোঁজখবর নিতে হবে সামনে এগোনোর আগে</t>
+  </si>
+  <si>
+    <t>আরাত্তুন আরো ভালা গরি হোছহবর লন ফরিবু সামনে আগাইবের আগে</t>
+  </si>
+  <si>
+    <t>এই সমস্যাটার জন্য আমরা সামনে এগোতে পারছি না</t>
+  </si>
+  <si>
+    <t>এই সমস্যা ইয়েনুর লাই আঁরা সামনে আগাইত ন পারির</t>
+  </si>
+  <si>
+    <t>আস্তে আস্তে আমরা একদম শেষের দিকে চলে আসছি</t>
+  </si>
+  <si>
+    <t>আস্তে আস্তে আঁরা এব্বেরে শেষুর দিকে চলি আইসসি</t>
+  </si>
+  <si>
+    <t>আর দু-একটা শব্দ লিখলেই আমাদের ডাটাসেট সম্পূর্ণ হয়ে যাবে</t>
+  </si>
+  <si>
+    <t>আর দুই-এক্কান শব্দ লেহিলিই আঁরার ডাটাসেট সম্পূর্ণ অই যাইবু</t>
+  </si>
+  <si>
+    <t>এখন যতটুকু হয়েছে সেটা নিয়ে আমাদের বাকি কাজ শুরু করে দিতে হবে</t>
+  </si>
+  <si>
+    <t>এহন যেদ্দুর অইয়্যি ইয়েন লই আরাত্তুন বাকি হাজ শুরু গরি দন ফরিবু</t>
+  </si>
+  <si>
+    <t>আমি আপাতত এতটুকু লিখলাম, যদি সময় থাকে বাকি শব্দগুলোও লিখব</t>
+  </si>
+  <si>
+    <t>আঁই আপাতত এদ্দুর লেহিলাম, যদি সময় থাহে বাকি শব্দ এগুনও লেইক্কুম</t>
   </si>
 </sst>
 </file>
@@ -25020,463 +25653,881 @@
       <c r="A1692" s="2" t="s">
         <v>3376</v>
       </c>
-      <c r="B1692" s="2"/>
+      <c r="B1692" s="2" t="s">
+        <v>3377</v>
+      </c>
     </row>
     <row r="1693" ht="25" customHeight="1" spans="1:2">
       <c r="A1693" s="2" t="s">
-        <v>3377</v>
-      </c>
-      <c r="B1693" s="2"/>
+        <v>3378</v>
+      </c>
+      <c r="B1693" s="2" t="s">
+        <v>3379</v>
+      </c>
     </row>
     <row r="1694" ht="25" customHeight="1" spans="1:2">
       <c r="A1694" s="2" t="s">
-        <v>3378</v>
-      </c>
-      <c r="B1694" s="2"/>
+        <v>3380</v>
+      </c>
+      <c r="B1694" s="2" t="s">
+        <v>3381</v>
+      </c>
     </row>
     <row r="1695" ht="25" customHeight="1" spans="1:2">
       <c r="A1695" s="2" t="s">
-        <v>3379</v>
-      </c>
-      <c r="B1695" s="2"/>
+        <v>3382</v>
+      </c>
+      <c r="B1695" s="2" t="s">
+        <v>3383</v>
+      </c>
     </row>
     <row r="1696" ht="25" customHeight="1" spans="1:2">
       <c r="A1696" s="2" t="s">
-        <v>3380</v>
-      </c>
-      <c r="B1696" s="2"/>
+        <v>3384</v>
+      </c>
+      <c r="B1696" s="2" t="s">
+        <v>3385</v>
+      </c>
     </row>
     <row r="1697" ht="25" customHeight="1" spans="1:2">
       <c r="A1697" s="2" t="s">
-        <v>3381</v>
-      </c>
-      <c r="B1697" s="2"/>
+        <v>3386</v>
+      </c>
+      <c r="B1697" s="2" t="s">
+        <v>3387</v>
+      </c>
     </row>
     <row r="1698" ht="25" customHeight="1" spans="1:2">
       <c r="A1698" s="2" t="s">
-        <v>3382</v>
-      </c>
-      <c r="B1698" s="2"/>
+        <v>3388</v>
+      </c>
+      <c r="B1698" s="2" t="s">
+        <v>3389</v>
+      </c>
     </row>
     <row r="1699" ht="25" customHeight="1" spans="1:2">
       <c r="A1699" s="2" t="s">
-        <v>3383</v>
-      </c>
-      <c r="B1699" s="2"/>
+        <v>3390</v>
+      </c>
+      <c r="B1699" s="2" t="s">
+        <v>3391</v>
+      </c>
     </row>
     <row r="1700" ht="25" customHeight="1" spans="1:2">
       <c r="A1700" s="2" t="s">
-        <v>3384</v>
-      </c>
-      <c r="B1700" s="2"/>
+        <v>3392</v>
+      </c>
+      <c r="B1700" s="2" t="s">
+        <v>3393</v>
+      </c>
     </row>
     <row r="1701" ht="25" customHeight="1" spans="1:2">
       <c r="A1701" s="2" t="s">
-        <v>3385</v>
-      </c>
-      <c r="B1701" s="2"/>
+        <v>3394</v>
+      </c>
+      <c r="B1701" s="2" t="s">
+        <v>3395</v>
+      </c>
     </row>
     <row r="1702" ht="25" customHeight="1" spans="1:2">
       <c r="A1702" s="2" t="s">
-        <v>3386</v>
-      </c>
-      <c r="B1702" s="2"/>
+        <v>3396</v>
+      </c>
+      <c r="B1702" s="2" t="s">
+        <v>3397</v>
+      </c>
     </row>
     <row r="1703" ht="25" customHeight="1" spans="1:2">
-      <c r="A1703" s="2"/>
-      <c r="B1703" s="2"/>
+      <c r="A1703" s="2" t="s">
+        <v>3398</v>
+      </c>
+      <c r="B1703" s="2" t="s">
+        <v>3399</v>
+      </c>
     </row>
     <row r="1704" ht="25" customHeight="1" spans="1:2">
-      <c r="A1704" s="2"/>
-      <c r="B1704" s="2"/>
+      <c r="A1704" s="2" t="s">
+        <v>3400</v>
+      </c>
+      <c r="B1704" s="2" t="s">
+        <v>3401</v>
+      </c>
     </row>
     <row r="1705" ht="25" customHeight="1" spans="1:2">
-      <c r="A1705" s="2"/>
-      <c r="B1705" s="2"/>
+      <c r="A1705" s="2" t="s">
+        <v>3402</v>
+      </c>
+      <c r="B1705" s="2" t="s">
+        <v>3403</v>
+      </c>
     </row>
     <row r="1706" ht="25" customHeight="1" spans="1:2">
-      <c r="A1706" s="2"/>
-      <c r="B1706" s="2"/>
+      <c r="A1706" s="2" t="s">
+        <v>3404</v>
+      </c>
+      <c r="B1706" s="2" t="s">
+        <v>3405</v>
+      </c>
     </row>
     <row r="1707" ht="25" customHeight="1" spans="1:2">
-      <c r="A1707" s="2"/>
-      <c r="B1707" s="2"/>
+      <c r="A1707" s="2" t="s">
+        <v>3406</v>
+      </c>
+      <c r="B1707" s="2" t="s">
+        <v>3407</v>
+      </c>
     </row>
     <row r="1708" ht="25" customHeight="1" spans="1:2">
-      <c r="A1708" s="2"/>
-      <c r="B1708" s="2"/>
+      <c r="A1708" s="2" t="s">
+        <v>3408</v>
+      </c>
+      <c r="B1708" s="2" t="s">
+        <v>3409</v>
+      </c>
     </row>
     <row r="1709" ht="25" customHeight="1" spans="1:2">
-      <c r="A1709" s="2"/>
-      <c r="B1709" s="2"/>
+      <c r="A1709" s="2" t="s">
+        <v>3410</v>
+      </c>
+      <c r="B1709" s="2" t="s">
+        <v>3411</v>
+      </c>
     </row>
     <row r="1710" ht="25" customHeight="1" spans="1:2">
-      <c r="A1710" s="2"/>
-      <c r="B1710" s="2"/>
+      <c r="A1710" s="2" t="s">
+        <v>3412</v>
+      </c>
+      <c r="B1710" s="2" t="s">
+        <v>3413</v>
+      </c>
     </row>
     <row r="1711" ht="25" customHeight="1" spans="1:2">
-      <c r="A1711" s="2"/>
-      <c r="B1711" s="2"/>
+      <c r="A1711" s="2" t="s">
+        <v>3414</v>
+      </c>
+      <c r="B1711" s="2" t="s">
+        <v>3415</v>
+      </c>
     </row>
     <row r="1712" ht="25" customHeight="1" spans="1:2">
-      <c r="A1712" s="2"/>
-      <c r="B1712" s="2"/>
+      <c r="A1712" s="2" t="s">
+        <v>3416</v>
+      </c>
+      <c r="B1712" s="2" t="s">
+        <v>3417</v>
+      </c>
     </row>
     <row r="1713" ht="25" customHeight="1" spans="1:2">
-      <c r="A1713" s="2"/>
-      <c r="B1713" s="2"/>
+      <c r="A1713" s="2" t="s">
+        <v>3418</v>
+      </c>
+      <c r="B1713" s="2" t="s">
+        <v>3419</v>
+      </c>
     </row>
     <row r="1714" ht="25" customHeight="1" spans="1:2">
-      <c r="A1714" s="2"/>
-      <c r="B1714" s="2"/>
+      <c r="A1714" s="2" t="s">
+        <v>3420</v>
+      </c>
+      <c r="B1714" s="2" t="s">
+        <v>3421</v>
+      </c>
     </row>
     <row r="1715" ht="25" customHeight="1" spans="1:2">
-      <c r="A1715" s="2"/>
-      <c r="B1715" s="2"/>
+      <c r="A1715" s="2" t="s">
+        <v>3422</v>
+      </c>
+      <c r="B1715" s="2" t="s">
+        <v>3423</v>
+      </c>
     </row>
     <row r="1716" ht="25" customHeight="1" spans="1:2">
-      <c r="A1716" s="2"/>
-      <c r="B1716" s="2"/>
+      <c r="A1716" s="2" t="s">
+        <v>3424</v>
+      </c>
+      <c r="B1716" s="2" t="s">
+        <v>3425</v>
+      </c>
     </row>
     <row r="1717" ht="25" customHeight="1" spans="1:2">
-      <c r="A1717" s="2"/>
-      <c r="B1717" s="2"/>
+      <c r="A1717" s="2" t="s">
+        <v>3426</v>
+      </c>
+      <c r="B1717" s="2" t="s">
+        <v>3427</v>
+      </c>
     </row>
     <row r="1718" ht="25" customHeight="1" spans="1:2">
-      <c r="A1718" s="2"/>
-      <c r="B1718" s="2"/>
+      <c r="A1718" s="2" t="s">
+        <v>3428</v>
+      </c>
+      <c r="B1718" s="2" t="s">
+        <v>3429</v>
+      </c>
     </row>
     <row r="1719" ht="25" customHeight="1" spans="1:2">
-      <c r="A1719" s="2"/>
-      <c r="B1719" s="2"/>
+      <c r="A1719" s="2" t="s">
+        <v>3430</v>
+      </c>
+      <c r="B1719" s="2" t="s">
+        <v>3431</v>
+      </c>
     </row>
     <row r="1720" ht="25" customHeight="1" spans="1:2">
-      <c r="A1720" s="2"/>
-      <c r="B1720" s="2"/>
+      <c r="A1720" s="2" t="s">
+        <v>3432</v>
+      </c>
+      <c r="B1720" s="2" t="s">
+        <v>3433</v>
+      </c>
     </row>
     <row r="1721" ht="25" customHeight="1" spans="1:2">
-      <c r="A1721" s="2"/>
-      <c r="B1721" s="2"/>
+      <c r="A1721" s="2" t="s">
+        <v>3434</v>
+      </c>
+      <c r="B1721" s="2" t="s">
+        <v>3435</v>
+      </c>
     </row>
     <row r="1722" ht="25" customHeight="1" spans="1:2">
-      <c r="A1722" s="2"/>
-      <c r="B1722" s="2"/>
+      <c r="A1722" s="2" t="s">
+        <v>3436</v>
+      </c>
+      <c r="B1722" s="2" t="s">
+        <v>3437</v>
+      </c>
     </row>
     <row r="1723" ht="25" customHeight="1" spans="1:2">
-      <c r="A1723" s="2"/>
-      <c r="B1723" s="2"/>
+      <c r="A1723" s="2" t="s">
+        <v>3438</v>
+      </c>
+      <c r="B1723" s="2" t="s">
+        <v>3439</v>
+      </c>
     </row>
     <row r="1724" ht="25" customHeight="1" spans="1:2">
-      <c r="A1724" s="2"/>
-      <c r="B1724" s="2"/>
+      <c r="A1724" s="2" t="s">
+        <v>3440</v>
+      </c>
+      <c r="B1724" s="2" t="s">
+        <v>3441</v>
+      </c>
     </row>
     <row r="1725" ht="25" customHeight="1" spans="1:2">
-      <c r="A1725" s="2"/>
-      <c r="B1725" s="2"/>
+      <c r="A1725" s="2" t="s">
+        <v>3442</v>
+      </c>
+      <c r="B1725" s="2" t="s">
+        <v>3443</v>
+      </c>
     </row>
     <row r="1726" ht="25" customHeight="1" spans="1:2">
-      <c r="A1726" s="2"/>
-      <c r="B1726" s="2"/>
+      <c r="A1726" s="2" t="s">
+        <v>3444</v>
+      </c>
+      <c r="B1726" s="2" t="s">
+        <v>3445</v>
+      </c>
     </row>
     <row r="1727" ht="25" customHeight="1" spans="1:2">
-      <c r="A1727" s="2"/>
-      <c r="B1727" s="2"/>
+      <c r="A1727" s="2" t="s">
+        <v>3446</v>
+      </c>
+      <c r="B1727" s="2" t="s">
+        <v>3447</v>
+      </c>
     </row>
     <row r="1728" ht="25" customHeight="1" spans="1:2">
-      <c r="A1728" s="2"/>
-      <c r="B1728" s="2"/>
+      <c r="A1728" s="2" t="s">
+        <v>3448</v>
+      </c>
+      <c r="B1728" s="2" t="s">
+        <v>3449</v>
+      </c>
     </row>
     <row r="1729" ht="25" customHeight="1" spans="1:2">
-      <c r="A1729" s="2"/>
-      <c r="B1729" s="2"/>
+      <c r="A1729" s="2" t="s">
+        <v>3450</v>
+      </c>
+      <c r="B1729" s="2" t="s">
+        <v>3451</v>
+      </c>
     </row>
     <row r="1730" ht="25" customHeight="1" spans="1:2">
-      <c r="A1730" s="2"/>
-      <c r="B1730" s="2"/>
+      <c r="A1730" s="2" t="s">
+        <v>3452</v>
+      </c>
+      <c r="B1730" s="2" t="s">
+        <v>3453</v>
+      </c>
     </row>
     <row r="1731" ht="25" customHeight="1" spans="1:2">
-      <c r="A1731" s="2"/>
-      <c r="B1731" s="2"/>
+      <c r="A1731" s="2" t="s">
+        <v>3454</v>
+      </c>
+      <c r="B1731" s="2" t="s">
+        <v>3455</v>
+      </c>
     </row>
     <row r="1732" ht="25" customHeight="1" spans="1:2">
-      <c r="A1732" s="2"/>
-      <c r="B1732" s="2"/>
+      <c r="A1732" s="2" t="s">
+        <v>3456</v>
+      </c>
+      <c r="B1732" s="2" t="s">
+        <v>3457</v>
+      </c>
     </row>
     <row r="1733" ht="25" customHeight="1" spans="1:2">
-      <c r="A1733" s="2"/>
-      <c r="B1733" s="2"/>
+      <c r="A1733" s="2" t="s">
+        <v>3458</v>
+      </c>
+      <c r="B1733" s="2" t="s">
+        <v>3459</v>
+      </c>
     </row>
     <row r="1734" ht="25" customHeight="1" spans="1:2">
-      <c r="A1734" s="2"/>
-      <c r="B1734" s="2"/>
+      <c r="A1734" s="2" t="s">
+        <v>3460</v>
+      </c>
+      <c r="B1734" s="2" t="s">
+        <v>3461</v>
+      </c>
     </row>
     <row r="1735" ht="25" customHeight="1" spans="1:2">
-      <c r="A1735" s="2"/>
-      <c r="B1735" s="2"/>
+      <c r="A1735" s="2" t="s">
+        <v>3462</v>
+      </c>
+      <c r="B1735" s="2" t="s">
+        <v>3463</v>
+      </c>
     </row>
     <row r="1736" ht="25" customHeight="1" spans="1:2">
-      <c r="A1736" s="2"/>
-      <c r="B1736" s="2"/>
+      <c r="A1736" s="2" t="s">
+        <v>3464</v>
+      </c>
+      <c r="B1736" s="2" t="s">
+        <v>3465</v>
+      </c>
     </row>
     <row r="1737" ht="25" customHeight="1" spans="1:2">
-      <c r="A1737" s="2"/>
-      <c r="B1737" s="2"/>
+      <c r="A1737" s="2" t="s">
+        <v>3466</v>
+      </c>
+      <c r="B1737" s="2" t="s">
+        <v>3467</v>
+      </c>
     </row>
     <row r="1738" ht="25" customHeight="1" spans="1:2">
-      <c r="A1738" s="2"/>
-      <c r="B1738" s="2"/>
+      <c r="A1738" s="2" t="s">
+        <v>3468</v>
+      </c>
+      <c r="B1738" s="2" t="s">
+        <v>3469</v>
+      </c>
     </row>
     <row r="1739" ht="25" customHeight="1" spans="1:2">
-      <c r="A1739" s="2"/>
-      <c r="B1739" s="2"/>
+      <c r="A1739" s="2" t="s">
+        <v>3470</v>
+      </c>
+      <c r="B1739" s="2" t="s">
+        <v>3471</v>
+      </c>
     </row>
     <row r="1740" ht="25" customHeight="1" spans="1:2">
-      <c r="A1740" s="2"/>
-      <c r="B1740" s="2"/>
+      <c r="A1740" s="2" t="s">
+        <v>3472</v>
+      </c>
+      <c r="B1740" s="2" t="s">
+        <v>3473</v>
+      </c>
     </row>
     <row r="1741" ht="25" customHeight="1" spans="1:2">
-      <c r="A1741" s="2"/>
-      <c r="B1741" s="2"/>
+      <c r="A1741" s="2" t="s">
+        <v>3474</v>
+      </c>
+      <c r="B1741" s="2" t="s">
+        <v>3475</v>
+      </c>
     </row>
     <row r="1742" ht="25" customHeight="1" spans="1:2">
-      <c r="A1742" s="2"/>
-      <c r="B1742" s="2"/>
+      <c r="A1742" s="2" t="s">
+        <v>3476</v>
+      </c>
+      <c r="B1742" s="2" t="s">
+        <v>3477</v>
+      </c>
     </row>
     <row r="1743" ht="25" customHeight="1" spans="1:2">
-      <c r="A1743" s="2"/>
-      <c r="B1743" s="2"/>
+      <c r="A1743" s="2" t="s">
+        <v>3478</v>
+      </c>
+      <c r="B1743" s="2" t="s">
+        <v>3479</v>
+      </c>
     </row>
     <row r="1744" ht="25" customHeight="1" spans="1:2">
-      <c r="A1744" s="2"/>
-      <c r="B1744" s="2"/>
+      <c r="A1744" s="2" t="s">
+        <v>3480</v>
+      </c>
+      <c r="B1744" s="2" t="s">
+        <v>3481</v>
+      </c>
     </row>
     <row r="1745" ht="25" customHeight="1" spans="1:2">
-      <c r="A1745" s="2"/>
-      <c r="B1745" s="2"/>
+      <c r="A1745" s="2" t="s">
+        <v>3482</v>
+      </c>
+      <c r="B1745" s="2" t="s">
+        <v>3483</v>
+      </c>
     </row>
     <row r="1746" ht="25" customHeight="1" spans="1:2">
-      <c r="A1746" s="2"/>
-      <c r="B1746" s="2"/>
+      <c r="A1746" s="2" t="s">
+        <v>3484</v>
+      </c>
+      <c r="B1746" s="2" t="s">
+        <v>3485</v>
+      </c>
     </row>
     <row r="1747" ht="25" customHeight="1" spans="1:2">
-      <c r="A1747" s="2"/>
-      <c r="B1747" s="2"/>
+      <c r="A1747" s="2" t="s">
+        <v>3486</v>
+      </c>
+      <c r="B1747" s="2" t="s">
+        <v>3487</v>
+      </c>
     </row>
     <row r="1748" ht="25" customHeight="1" spans="1:2">
-      <c r="A1748" s="2"/>
-      <c r="B1748" s="2"/>
+      <c r="A1748" s="2" t="s">
+        <v>3488</v>
+      </c>
+      <c r="B1748" s="2" t="s">
+        <v>3489</v>
+      </c>
     </row>
     <row r="1749" ht="25" customHeight="1" spans="1:2">
-      <c r="A1749" s="2"/>
-      <c r="B1749" s="2"/>
+      <c r="A1749" s="2" t="s">
+        <v>3490</v>
+      </c>
+      <c r="B1749" s="2" t="s">
+        <v>3491</v>
+      </c>
     </row>
     <row r="1750" ht="25" customHeight="1" spans="1:2">
-      <c r="A1750" s="2"/>
-      <c r="B1750" s="2"/>
+      <c r="A1750" s="2" t="s">
+        <v>3492</v>
+      </c>
+      <c r="B1750" s="2" t="s">
+        <v>3493</v>
+      </c>
     </row>
     <row r="1751" ht="25" customHeight="1" spans="1:2">
-      <c r="A1751" s="2"/>
-      <c r="B1751" s="2"/>
+      <c r="A1751" s="2" t="s">
+        <v>3494</v>
+      </c>
+      <c r="B1751" s="2" t="s">
+        <v>3495</v>
+      </c>
     </row>
     <row r="1752" ht="25" customHeight="1" spans="1:2">
-      <c r="A1752" s="2"/>
-      <c r="B1752" s="2"/>
+      <c r="A1752" s="2" t="s">
+        <v>3496</v>
+      </c>
+      <c r="B1752" s="2" t="s">
+        <v>3497</v>
+      </c>
     </row>
     <row r="1753" ht="25" customHeight="1" spans="1:2">
-      <c r="A1753" s="2"/>
-      <c r="B1753" s="2"/>
+      <c r="A1753" s="2" t="s">
+        <v>3498</v>
+      </c>
+      <c r="B1753" s="2" t="s">
+        <v>3499</v>
+      </c>
     </row>
     <row r="1754" ht="25" customHeight="1" spans="1:2">
-      <c r="A1754" s="2"/>
-      <c r="B1754" s="2"/>
+      <c r="A1754" s="2" t="s">
+        <v>3500</v>
+      </c>
+      <c r="B1754" s="2" t="s">
+        <v>3501</v>
+      </c>
     </row>
     <row r="1755" ht="25" customHeight="1" spans="1:2">
-      <c r="A1755" s="2"/>
-      <c r="B1755" s="2"/>
+      <c r="A1755" s="2" t="s">
+        <v>3502</v>
+      </c>
+      <c r="B1755" s="2" t="s">
+        <v>3503</v>
+      </c>
     </row>
     <row r="1756" ht="25" customHeight="1" spans="1:2">
-      <c r="A1756" s="2"/>
-      <c r="B1756" s="2"/>
+      <c r="A1756" s="2" t="s">
+        <v>3504</v>
+      </c>
+      <c r="B1756" s="2" t="s">
+        <v>3505</v>
+      </c>
     </row>
     <row r="1757" ht="25" customHeight="1" spans="1:2">
-      <c r="A1757" s="2"/>
-      <c r="B1757" s="2"/>
+      <c r="A1757" s="2" t="s">
+        <v>3506</v>
+      </c>
+      <c r="B1757" s="2" t="s">
+        <v>3507</v>
+      </c>
     </row>
     <row r="1758" ht="25" customHeight="1" spans="1:2">
-      <c r="A1758" s="2"/>
-      <c r="B1758" s="2"/>
+      <c r="A1758" s="2" t="s">
+        <v>3508</v>
+      </c>
+      <c r="B1758" s="2" t="s">
+        <v>3509</v>
+      </c>
     </row>
     <row r="1759" ht="25" customHeight="1" spans="1:2">
-      <c r="A1759" s="2"/>
-      <c r="B1759" s="2"/>
+      <c r="A1759" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="B1759" s="2" t="s">
+        <v>3511</v>
+      </c>
     </row>
     <row r="1760" ht="25" customHeight="1" spans="1:2">
-      <c r="A1760" s="2"/>
-      <c r="B1760" s="2"/>
+      <c r="A1760" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="B1760" s="2" t="s">
+        <v>3513</v>
+      </c>
     </row>
     <row r="1761" ht="25" customHeight="1" spans="1:2">
-      <c r="A1761" s="2"/>
-      <c r="B1761" s="2"/>
+      <c r="A1761" s="2" t="s">
+        <v>3514</v>
+      </c>
+      <c r="B1761" s="2" t="s">
+        <v>3515</v>
+      </c>
     </row>
     <row r="1762" ht="25" customHeight="1" spans="1:2">
-      <c r="A1762" s="2"/>
-      <c r="B1762" s="2"/>
+      <c r="A1762" s="2" t="s">
+        <v>3516</v>
+      </c>
+      <c r="B1762" s="2" t="s">
+        <v>3517</v>
+      </c>
     </row>
     <row r="1763" ht="25" customHeight="1" spans="1:2">
-      <c r="A1763" s="2"/>
-      <c r="B1763" s="2"/>
+      <c r="A1763" s="2" t="s">
+        <v>3518</v>
+      </c>
+      <c r="B1763" s="2" t="s">
+        <v>3519</v>
+      </c>
     </row>
     <row r="1764" ht="25" customHeight="1" spans="1:2">
-      <c r="A1764" s="2"/>
-      <c r="B1764" s="2"/>
+      <c r="A1764" s="2" t="s">
+        <v>3520</v>
+      </c>
+      <c r="B1764" s="2" t="s">
+        <v>3521</v>
+      </c>
     </row>
     <row r="1765" ht="25" customHeight="1" spans="1:2">
-      <c r="A1765" s="2"/>
-      <c r="B1765" s="2"/>
+      <c r="A1765" s="2" t="s">
+        <v>3522</v>
+      </c>
+      <c r="B1765" s="2" t="s">
+        <v>3523</v>
+      </c>
     </row>
     <row r="1766" ht="25" customHeight="1" spans="1:2">
-      <c r="A1766" s="2"/>
-      <c r="B1766" s="2"/>
+      <c r="A1766" s="2" t="s">
+        <v>3524</v>
+      </c>
+      <c r="B1766" s="2" t="s">
+        <v>3525</v>
+      </c>
     </row>
     <row r="1767" ht="25" customHeight="1" spans="1:2">
-      <c r="A1767" s="2"/>
-      <c r="B1767" s="2"/>
+      <c r="A1767" s="2" t="s">
+        <v>3526</v>
+      </c>
+      <c r="B1767" s="2" t="s">
+        <v>3527</v>
+      </c>
     </row>
     <row r="1768" ht="25" customHeight="1" spans="1:2">
-      <c r="A1768" s="2"/>
-      <c r="B1768" s="2"/>
+      <c r="A1768" s="2" t="s">
+        <v>3528</v>
+      </c>
+      <c r="B1768" s="2" t="s">
+        <v>3529</v>
+      </c>
     </row>
     <row r="1769" ht="25" customHeight="1" spans="1:2">
-      <c r="A1769" s="2"/>
-      <c r="B1769" s="2"/>
+      <c r="A1769" s="2" t="s">
+        <v>3530</v>
+      </c>
+      <c r="B1769" s="2" t="s">
+        <v>3531</v>
+      </c>
     </row>
     <row r="1770" ht="25" customHeight="1" spans="1:2">
-      <c r="A1770" s="2"/>
-      <c r="B1770" s="2"/>
+      <c r="A1770" s="2" t="s">
+        <v>3532</v>
+      </c>
+      <c r="B1770" s="2" t="s">
+        <v>3533</v>
+      </c>
     </row>
     <row r="1771" ht="25" customHeight="1" spans="1:2">
-      <c r="A1771" s="2"/>
-      <c r="B1771" s="2"/>
+      <c r="A1771" s="2" t="s">
+        <v>3534</v>
+      </c>
+      <c r="B1771" s="2" t="s">
+        <v>3535</v>
+      </c>
     </row>
     <row r="1772" ht="25" customHeight="1" spans="1:2">
-      <c r="A1772" s="2"/>
-      <c r="B1772" s="2"/>
+      <c r="A1772" s="2" t="s">
+        <v>3536</v>
+      </c>
+      <c r="B1772" s="2" t="s">
+        <v>3537</v>
+      </c>
     </row>
     <row r="1773" ht="25" customHeight="1" spans="1:2">
-      <c r="A1773" s="2"/>
-      <c r="B1773" s="2"/>
+      <c r="A1773" s="2" t="s">
+        <v>3538</v>
+      </c>
+      <c r="B1773" s="2" t="s">
+        <v>3539</v>
+      </c>
     </row>
     <row r="1774" ht="25" customHeight="1" spans="1:2">
-      <c r="A1774" s="2"/>
-      <c r="B1774" s="2"/>
+      <c r="A1774" s="2" t="s">
+        <v>3540</v>
+      </c>
+      <c r="B1774" s="2" t="s">
+        <v>3541</v>
+      </c>
     </row>
     <row r="1775" ht="25" customHeight="1" spans="1:2">
-      <c r="A1775" s="2"/>
-      <c r="B1775" s="2"/>
+      <c r="A1775" s="2" t="s">
+        <v>3542</v>
+      </c>
+      <c r="B1775" s="2" t="s">
+        <v>3543</v>
+      </c>
     </row>
     <row r="1776" ht="25" customHeight="1" spans="1:2">
-      <c r="A1776" s="2"/>
-      <c r="B1776" s="2"/>
+      <c r="A1776" s="2" t="s">
+        <v>3544</v>
+      </c>
+      <c r="B1776" s="2" t="s">
+        <v>3545</v>
+      </c>
     </row>
     <row r="1777" ht="25" customHeight="1" spans="1:2">
-      <c r="A1777" s="2"/>
-      <c r="B1777" s="2"/>
+      <c r="A1777" s="2" t="s">
+        <v>3546</v>
+      </c>
+      <c r="B1777" s="2" t="s">
+        <v>3547</v>
+      </c>
     </row>
     <row r="1778" ht="25" customHeight="1" spans="1:2">
-      <c r="A1778" s="2"/>
-      <c r="B1778" s="2"/>
+      <c r="A1778" s="2" t="s">
+        <v>3548</v>
+      </c>
+      <c r="B1778" s="2" t="s">
+        <v>3549</v>
+      </c>
     </row>
     <row r="1779" ht="25" customHeight="1" spans="1:2">
-      <c r="A1779" s="2"/>
-      <c r="B1779" s="2"/>
+      <c r="A1779" s="2" t="s">
+        <v>3550</v>
+      </c>
+      <c r="B1779" s="2" t="s">
+        <v>3551</v>
+      </c>
     </row>
     <row r="1780" ht="25" customHeight="1" spans="1:2">
-      <c r="A1780" s="2"/>
-      <c r="B1780" s="2"/>
+      <c r="A1780" s="2" t="s">
+        <v>3552</v>
+      </c>
+      <c r="B1780" s="2" t="s">
+        <v>3553</v>
+      </c>
     </row>
     <row r="1781" ht="25" customHeight="1" spans="1:2">
-      <c r="A1781" s="2"/>
-      <c r="B1781" s="2"/>
+      <c r="A1781" s="2" t="s">
+        <v>3554</v>
+      </c>
+      <c r="B1781" s="2" t="s">
+        <v>3555</v>
+      </c>
     </row>
     <row r="1782" ht="25" customHeight="1" spans="1:2">
-      <c r="A1782" s="2"/>
-      <c r="B1782" s="2"/>
+      <c r="A1782" s="2" t="s">
+        <v>3556</v>
+      </c>
+      <c r="B1782" s="2" t="s">
+        <v>3557</v>
+      </c>
     </row>
     <row r="1783" ht="25" customHeight="1" spans="1:2">
-      <c r="A1783" s="2"/>
-      <c r="B1783" s="2"/>
+      <c r="A1783" s="2" t="s">
+        <v>3558</v>
+      </c>
+      <c r="B1783" s="2" t="s">
+        <v>3559</v>
+      </c>
     </row>
     <row r="1784" ht="25" customHeight="1" spans="1:2">
-      <c r="A1784" s="2"/>
-      <c r="B1784" s="2"/>
+      <c r="A1784" s="2" t="s">
+        <v>3560</v>
+      </c>
+      <c r="B1784" s="2" t="s">
+        <v>3561</v>
+      </c>
     </row>
     <row r="1785" ht="25" customHeight="1" spans="1:2">
-      <c r="A1785" s="2"/>
-      <c r="B1785" s="2"/>
+      <c r="A1785" s="2" t="s">
+        <v>3562</v>
+      </c>
+      <c r="B1785" s="2" t="s">
+        <v>3563</v>
+      </c>
     </row>
     <row r="1786" ht="25" customHeight="1" spans="1:2">
-      <c r="A1786" s="2"/>
-      <c r="B1786" s="2"/>
+      <c r="A1786" s="2" t="s">
+        <v>3564</v>
+      </c>
+      <c r="B1786" s="2" t="s">
+        <v>3565</v>
+      </c>
     </row>
     <row r="1787" ht="25" customHeight="1" spans="1:2">
-      <c r="A1787" s="2"/>
-      <c r="B1787" s="2"/>
+      <c r="A1787" s="2" t="s">
+        <v>3566</v>
+      </c>
+      <c r="B1787" s="2" t="s">
+        <v>3567</v>
+      </c>
     </row>
     <row r="1788" ht="25" customHeight="1" spans="1:2">
-      <c r="A1788" s="2"/>
-      <c r="B1788" s="2"/>
+      <c r="A1788" s="2" t="s">
+        <v>3568</v>
+      </c>
+      <c r="B1788" s="2" t="s">
+        <v>3569</v>
+      </c>
     </row>
     <row r="1789" ht="25" customHeight="1" spans="1:2">
-      <c r="A1789" s="2"/>
-      <c r="B1789" s="2"/>
+      <c r="A1789" s="2" t="s">
+        <v>3570</v>
+      </c>
+      <c r="B1789" s="2" t="s">
+        <v>3571</v>
+      </c>
     </row>
     <row r="1790" ht="25" customHeight="1" spans="1:2">
-      <c r="A1790" s="2"/>
-      <c r="B1790" s="2"/>
+      <c r="A1790" s="2" t="s">
+        <v>3572</v>
+      </c>
+      <c r="B1790" s="2" t="s">
+        <v>3573</v>
+      </c>
     </row>
     <row r="1791" ht="25" customHeight="1" spans="1:2">
-      <c r="A1791" s="2"/>
-      <c r="B1791" s="2"/>
+      <c r="A1791" s="2" t="s">
+        <v>3574</v>
+      </c>
+      <c r="B1791" s="2" t="s">
+        <v>3575</v>
+      </c>
     </row>
     <row r="1792" ht="25" customHeight="1" spans="1:2">
-      <c r="A1792" s="2"/>
-      <c r="B1792" s="2"/>
+      <c r="A1792" s="2" t="s">
+        <v>3576</v>
+      </c>
+      <c r="B1792" s="2" t="s">
+        <v>3577</v>
+      </c>
     </row>
     <row r="1793" ht="25" customHeight="1" spans="1:2">
-      <c r="A1793" s="2"/>
-      <c r="B1793" s="2"/>
+      <c r="A1793" s="2" t="s">
+        <v>3578</v>
+      </c>
+      <c r="B1793" s="2" t="s">
+        <v>3579</v>
+      </c>
     </row>
     <row r="1794" ht="25" customHeight="1" spans="1:2">
-      <c r="A1794" s="2"/>
-      <c r="B1794" s="2"/>
+      <c r="A1794" s="2" t="s">
+        <v>3580</v>
+      </c>
+      <c r="B1794" s="2" t="s">
+        <v>3581</v>
+      </c>
     </row>
     <row r="1795" ht="25" customHeight="1" spans="1:2">
-      <c r="A1795" s="2"/>
-      <c r="B1795" s="2"/>
+      <c r="A1795" s="2" t="s">
+        <v>3582</v>
+      </c>
+      <c r="B1795" s="2" t="s">
+        <v>3583</v>
+      </c>
     </row>
     <row r="1796" ht="25" customHeight="1" spans="1:2">
-      <c r="A1796" s="2"/>
-      <c r="B1796" s="2"/>
+      <c r="A1796" s="2" t="s">
+        <v>3584</v>
+      </c>
+      <c r="B1796" s="2" t="s">
+        <v>3585</v>
+      </c>
     </row>
     <row r="1797" ht="25" customHeight="1" spans="1:2">
-      <c r="A1797" s="2"/>
-      <c r="B1797" s="2"/>
+      <c r="A1797" s="2" t="s">
+        <v>3586</v>
+      </c>
+      <c r="B1797" s="2" t="s">
+        <v>3587</v>
+      </c>
     </row>
     <row r="1798" ht="25" customHeight="1" spans="1:2">
-      <c r="A1798" s="2"/>
-      <c r="B1798" s="2"/>
+      <c r="A1798" s="2" t="s">
+        <v>3588</v>
+      </c>
+      <c r="B1798" s="2" t="s">
+        <v>3589</v>
+      </c>
     </row>
     <row r="1799" ht="25" customHeight="1" spans="1:2">
-      <c r="A1799" s="2"/>
-      <c r="B1799" s="2"/>
+      <c r="A1799" s="2" t="s">
+        <v>3590</v>
+      </c>
+      <c r="B1799" s="2" t="s">
+        <v>3591</v>
+      </c>
     </row>
     <row r="1800" ht="25" customHeight="1" spans="1:2">
-      <c r="A1800" s="2"/>
-      <c r="B1800" s="2"/>
+      <c r="A1800" s="2" t="s">
+        <v>3592</v>
+      </c>
+      <c r="B1800" s="2" t="s">
+        <v>3593</v>
+      </c>
     </row>
     <row r="1801" ht="25" customHeight="1" spans="1:2">
-      <c r="A1801" s="2"/>
-      <c r="B1801" s="2"/>
+      <c r="A1801" s="2" t="s">
+        <v>3594</v>
+      </c>
+      <c r="B1801" s="2" t="s">
+        <v>3595</v>
+      </c>
     </row>
     <row r="1802" ht="25" customHeight="1" spans="1:2">
       <c r="A1802" s="2"/>

</xml_diff>